<commit_message>
feat: preserve pre-possession rents and total amount paid in history and flat details modal, and generate final 3 spreadsheets
</commit_message>
<xml_diff>
--- a/Tower_A_Inventory_3_Possession_Renewal.xlsx
+++ b/Tower_A_Inventory_3_Possession_Renewal.xlsx
@@ -1312,7 +1312,7 @@
         <v>5500000</v>
       </c>
       <c r="M2" t="str">
-        <v>Flat A-204: Pre-Possession Contract (100mo @ ₹16000/mo, Total: ₹16,00,000) expired/renewed to Post-Possession Rate (@ ₹9,000/mo)</v>
+        <v>Flat A-204: Pre-Possession Contract (100mo @ ₹16000/mo, Total Disbursed: ₹16,00,000) renewed to Post-Possession Rate (@ ₹9,000/mo)</v>
       </c>
     </row>
     <row r="3">
@@ -1338,7 +1338,7 @@
         <v>possession_renewal</v>
       </c>
       <c r="H3">
-        <v>1738600</v>
+        <v>928000</v>
       </c>
       <c r="I3" t="str">
         <v>Aman Sharma</v>
@@ -1353,7 +1353,7 @@
         <v>5500000</v>
       </c>
       <c r="M3" t="str">
-        <v>Flat A-212: Pre-Possession Contract (100mo @ ₹16000/mo, Total: ₹17,38,600) expired/renewed to Post-Possession Rate (@ ₹11,000/mo)</v>
+        <v>Flat A-212: Pre-Possession Contract (100mo @ ₹16000/mo, Total Disbursed: ₹9,28,000) renewed to Post-Possession Rate (@ ₹11,000/mo)</v>
       </c>
     </row>
     <row r="4">
@@ -1394,7 +1394,7 @@
         <v>5500000</v>
       </c>
       <c r="M4" t="str">
-        <v>Flat A-305: Pre-Possession Contract (91mo @ ₹16000/mo, Total: ₹14,56,000) expired/renewed to Post-Possession Rate (@ ₹11,000/mo)</v>
+        <v>Flat A-305: Pre-Possession Contract (91mo @ ₹16000/mo, Total Disbursed: ₹14,56,000) renewed to Post-Possession Rate (@ ₹11,000/mo)</v>
       </c>
     </row>
     <row r="5">
@@ -1420,7 +1420,7 @@
         <v>possession_renewal</v>
       </c>
       <c r="H5">
-        <v>1732000</v>
+        <v>960000</v>
       </c>
       <c r="I5" t="str">
         <v>Namita Jain</v>
@@ -1435,7 +1435,7 @@
         <v>5500000</v>
       </c>
       <c r="M5" t="str">
-        <v>Flat A-312: Pre-Possession Contract (100mo @ ₹16000/mo, Total: ₹17,32,000) expired/renewed to Post-Possession Rate (@ ₹11,000/mo)</v>
+        <v>Flat A-312: Pre-Possession Contract (100mo @ ₹16000/mo, Total Disbursed: ₹9,60,000) renewed to Post-Possession Rate (@ ₹11,000/mo)</v>
       </c>
     </row>
     <row r="6">
@@ -1476,7 +1476,7 @@
         <v>5500000</v>
       </c>
       <c r="M6" t="str">
-        <v>Flat A-402: Pre-Possession Contract (100mo @ ₹22000/mo, Total: ₹22,00,000) expired/renewed to Post-Possession Rate (@ ₹11,000/mo)</v>
+        <v>Flat A-402: Pre-Possession Contract (100mo @ ₹22000/mo, Total Disbursed: ₹22,00,000) renewed to Post-Possession Rate (@ ₹11,000/mo)</v>
       </c>
     </row>
     <row r="7">
@@ -1517,7 +1517,7 @@
         <v>5500000</v>
       </c>
       <c r="M7" t="str">
-        <v>Flat A-403: Pre-Possession Contract (100mo @ ₹16000/mo, Total: ₹16,00,000) expired/renewed to Post-Possession Rate (@ ₹12,000/mo)</v>
+        <v>Flat A-403: Pre-Possession Contract (100mo @ ₹16000/mo, Total Disbursed: ₹16,00,000) renewed to Post-Possession Rate (@ ₹12,000/mo)</v>
       </c>
     </row>
     <row r="8">
@@ -1543,7 +1543,7 @@
         <v>possession_renewal</v>
       </c>
       <c r="H8">
-        <v>1716000</v>
+        <v>672000</v>
       </c>
       <c r="I8" t="str">
         <v>Geeta Giri</v>
@@ -1558,7 +1558,7 @@
         <v>5500000</v>
       </c>
       <c r="M8" t="str">
-        <v>Flat A-413: Pre-Possession Contract (100mo @ ₹16000/mo, Total: ₹17,16,000) expired/renewed to Post-Possession Rate (@ ₹16,000/mo)</v>
+        <v>Flat A-413: Pre-Possession Contract (100mo @ ₹16000/mo, Total Disbursed: ₹6,72,000) renewed to Post-Possession Rate (@ ₹16,000/mo)</v>
       </c>
     </row>
     <row r="9">
@@ -1584,7 +1584,7 @@
         <v>possession_renewal</v>
       </c>
       <c r="H9">
-        <v>1600000</v>
+        <v>672000</v>
       </c>
       <c r="I9" t="str">
         <v>Veena Sahani</v>
@@ -1599,7 +1599,7 @@
         <v>5500000</v>
       </c>
       <c r="M9" t="str">
-        <v>Flat A-507: Pre-Possession Contract (100mo @ ₹16000/mo, Total: ₹16,00,000) expired/renewed to Post-Possession Rate (@ ₹16,000/mo)</v>
+        <v>Flat A-507: Pre-Possession Contract (100mo @ ₹16000/mo, Total Disbursed: ₹6,72,000) renewed to Post-Possession Rate (@ ₹16,000/mo)</v>
       </c>
     </row>
     <row r="10">
@@ -1640,7 +1640,7 @@
         <v>5500000</v>
       </c>
       <c r="M10" t="str">
-        <v>Flat A-512: Pre-Possession Contract (100mo @ ₹22000/mo, Total: ₹22,00,000) expired/renewed to Post-Possession Rate (@ ₹11,000/mo)</v>
+        <v>Flat A-512: Pre-Possession Contract (100mo @ ₹22000/mo, Total Disbursed: ₹22,00,000) renewed to Post-Possession Rate (@ ₹11,000/mo)</v>
       </c>
     </row>
     <row r="11">
@@ -1681,7 +1681,7 @@
         <v>5500000</v>
       </c>
       <c r="M11" t="str">
-        <v>Flat A-612: Pre-Possession Contract (100mo @ ₹21500/mo, Total: ₹21,50,000) expired/renewed to Post-Possession Rate (@ ₹11,000/mo)</v>
+        <v>Flat A-612: Pre-Possession Contract (100mo @ ₹21500/mo, Total Disbursed: ₹21,50,000) renewed to Post-Possession Rate (@ ₹11,000/mo)</v>
       </c>
     </row>
     <row r="12">
@@ -1707,7 +1707,7 @@
         <v>possession_renewal</v>
       </c>
       <c r="H12">
-        <v>1716000</v>
+        <v>672000</v>
       </c>
       <c r="I12" t="str">
         <v>Sita Mathur</v>
@@ -1722,7 +1722,7 @@
         <v>5500000</v>
       </c>
       <c r="M12" t="str">
-        <v>Flat A-613: Pre-Possession Contract (100mo @ ₹16000/mo, Total: ₹17,16,000) expired/renewed to Post-Possession Rate (@ ₹10,000/mo)</v>
+        <v>Flat A-613: Pre-Possession Contract (100mo @ ₹16000/mo, Total Disbursed: ₹6,72,000) renewed to Post-Possession Rate (@ ₹10,000/mo)</v>
       </c>
     </row>
     <row r="13">
@@ -1763,7 +1763,7 @@
         <v>5500000</v>
       </c>
       <c r="M13" t="str">
-        <v>Flat A-806: Pre-Possession Contract (100mo @ ₹22000/mo, Total: ₹22,00,000) expired/renewed to Post-Possession Rate (@ ₹10,000/mo)</v>
+        <v>Flat A-806: Pre-Possession Contract (100mo @ ₹22000/mo, Total Disbursed: ₹22,00,000) renewed to Post-Possession Rate (@ ₹10,000/mo)</v>
       </c>
     </row>
     <row r="14">
@@ -1789,7 +1789,7 @@
         <v>possession_renewal</v>
       </c>
       <c r="H14">
-        <v>1767200</v>
+        <v>1457918</v>
       </c>
       <c r="I14" t="str">
         <v>Satyajeet Sharma</v>
@@ -1804,7 +1804,7 @@
         <v>5500000</v>
       </c>
       <c r="M14" t="str">
-        <v>Flat A-906: Pre-Possession Contract (100mo @ ₹20972/mo, Total: ₹17,67,200) expired/renewed to Post-Possession Rate (@ ₹20,972/mo)</v>
+        <v>Flat A-906: Pre-Possession Contract (100mo @ ₹20972/mo, Total Disbursed: ₹14,57,918) renewed to Post-Possession Rate (@ ₹20,972/mo)</v>
       </c>
     </row>
   </sheetData>

</xml_diff>